<commit_message>
updated tutorials, finished habituation
</commit_message>
<xml_diff>
--- a/apps_nicolo/LogicCircuits_4s_6r_HF_REINFORCE/LogicCircuits_4s_6r_HF_REINFORCE_SIL.xlsx
+++ b/apps_nicolo/LogicCircuits_4s_6r_HF_REINFORCE/LogicCircuits_4s_6r_HF_REINFORCE_SIL.xlsx
@@ -250,13 +250,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -288,7 +288,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
@@ -296,19 +296,13 @@
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="4" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -628,32 +622,32 @@
   <dimension ref="A1:Z14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="8" width="21.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="14.147857142857141" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="8" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="8" width="7.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="8" width="109.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="10" width="15.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="11" width="10.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="8" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="11" width="10.005" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="11" width="10.005" customWidth="1" bestFit="1"/>
-    <col min="12" max="12" style="11" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="13" max="13" style="11" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="14" max="14" style="8" width="178.005" customWidth="1" bestFit="1"/>
-    <col min="15" max="15" style="8" width="76.005" customWidth="1" bestFit="1"/>
-    <col min="16" max="16" style="11" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="17" max="17" style="11" width="10.005" customWidth="1" bestFit="1"/>
-    <col min="18" max="18" style="11" width="17.005" customWidth="1" bestFit="1"/>
-    <col min="19" max="19" style="11" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="20" max="20" style="11" width="22.005" customWidth="1" bestFit="1"/>
-    <col min="21" max="21" style="11" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="22" max="22" style="8" width="35.005" customWidth="1" bestFit="1"/>
-    <col min="23" max="23" style="8" width="80.005" customWidth="1" bestFit="1"/>
-    <col min="24" max="24" style="8" width="135.005" customWidth="1" bestFit="1"/>
-    <col min="25" max="25" style="8" width="19.005" customWidth="1" bestFit="1"/>
-    <col min="26" max="26" style="8" width="99.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="6" width="21.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="6" width="14.147857142857141" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="7" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="6" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="6" width="7.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="6" width="109.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="8" width="15.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="9" width="10.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="6" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="9" width="10.005" customWidth="1" bestFit="1"/>
+    <col min="11" max="11" style="9" width="10.005" customWidth="1" bestFit="1"/>
+    <col min="12" max="12" style="9" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="13" max="13" style="9" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="14" max="14" style="6" width="178.005" customWidth="1" bestFit="1"/>
+    <col min="15" max="15" style="6" width="76.005" customWidth="1" bestFit="1"/>
+    <col min="16" max="16" style="9" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="17" max="17" style="9" width="10.005" customWidth="1" bestFit="1"/>
+    <col min="18" max="18" style="9" width="17.005" customWidth="1" bestFit="1"/>
+    <col min="19" max="19" style="9" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="20" max="20" style="9" width="22.005" customWidth="1" bestFit="1"/>
+    <col min="21" max="21" style="9" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="22" max="22" style="6" width="35.005" customWidth="1" bestFit="1"/>
+    <col min="23" max="23" style="6" width="80.005" customWidth="1" bestFit="1"/>
+    <col min="24" max="24" style="6" width="135.005" customWidth="1" bestFit="1"/>
+    <col min="25" max="25" style="6" width="19.005" customWidth="1" bestFit="1"/>
+    <col min="26" max="26" style="6" width="99.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
@@ -743,7 +737,7 @@
       <c r="B2" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="5"/>
+      <c r="C2" s="4"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -815,7 +809,7 @@
       <c r="B3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="5"/>
+      <c r="C3" s="4"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -887,7 +881,7 @@
       <c r="B4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="5"/>
+      <c r="C4" s="4"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -959,7 +953,7 @@
       <c r="B5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="5"/>
+      <c r="C5" s="4"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -1031,7 +1025,7 @@
       <c r="B6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="5"/>
+      <c r="C6" s="4"/>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -1103,7 +1097,7 @@
       <c r="B7" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C7" s="5"/>
+      <c r="C7" s="4"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -1175,7 +1169,7 @@
       <c r="B8" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C8" s="5"/>
+      <c r="C8" s="4"/>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -1247,7 +1241,7 @@
       <c r="B9" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="5"/>
+      <c r="C9" s="4"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
@@ -1319,7 +1313,7 @@
       <c r="B10" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="5"/>
+      <c r="C10" s="4"/>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
@@ -1391,7 +1385,7 @@
       <c r="B11" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="5"/>
+      <c r="C11" s="4"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -1543,7 +1537,7 @@
       <c r="B13" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="4">
         <v>300</v>
       </c>
       <c r="D13" s="1" t="s">
@@ -1623,29 +1617,29 @@
       <c r="B14" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C14" s="6"/>
+      <c r="C14" s="5"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="7">
+      <c r="G14" s="3">
         <v>0.0001</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H14" s="4">
         <v>300</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="4">
         <v>5</v>
       </c>
-      <c r="K14" s="5">
+      <c r="K14" s="4">
         <v>1024</v>
       </c>
-      <c r="L14" s="5">
+      <c r="L14" s="4">
         <v>10240</v>
       </c>
-      <c r="M14" s="5">
+      <c r="M14" s="4">
         <v>128</v>
       </c>
       <c r="N14" s="1" t="s">
@@ -1654,22 +1648,22 @@
       <c r="O14" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="P14" s="5">
+      <c r="P14" s="4">
         <v>10</v>
       </c>
-      <c r="Q14" s="5">
-        <v>30</v>
-      </c>
-      <c r="R14" s="5">
+      <c r="Q14" s="4">
+        <v>30</v>
+      </c>
+      <c r="R14" s="4">
         <v>100</v>
       </c>
-      <c r="S14" s="5">
+      <c r="S14" s="4">
         <v>1000</v>
       </c>
-      <c r="T14" s="5">
+      <c r="T14" s="4">
         <v>1</v>
       </c>
-      <c r="U14" s="5">
+      <c r="U14" s="4">
         <v>16</v>
       </c>
       <c r="V14" s="1" t="s">

</xml_diff>